<commit_message>
debug det eq problem
</commit_message>
<xml_diff>
--- a/Starting_point.xlsx
+++ b/Starting_point.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fthcn\Desktop\Vaccine_Tender_Scheduling_Problem\Julia_Files\Github\Github\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A8FEE2-BE8F-4FE6-A73D-C8D61511F8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -153,7 +153,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="173" formatCode="0.000E+00"/>
+    <numFmt numFmtId="164" formatCode="0.000E+00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -225,7 +225,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -510,9 +510,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{942AD6D9-E2BE-4540-AD66-B6783F716305}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -523,7 +523,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -534,7 +534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -545,7 +545,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -556,7 +556,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -567,7 +567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -578,7 +578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -589,7 +589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -600,7 +600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -611,7 +611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -622,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -633,7 +633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -644,7 +644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -663,15 +663,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86710C76-81AC-48E5-8A5F-29B3CE6BD5DC}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="8.85546875" style="2"/>
     <col min="2" max="2" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.88671875" style="2"/>
-    <col min="5" max="5" width="16.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.85546875" style="2"/>
+    <col min="5" max="5" width="16.140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -688,7 +688,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -705,7 +705,7 @@
         <v>13299464</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -722,7 +722,7 @@
         <v>12505034</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -739,7 +739,7 @@
         <v>13547121</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -756,7 +756,7 @@
         <v>6547121</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -773,7 +773,7 @@
         <v>90279149</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -790,7 +790,7 @@
         <v>180177056</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -807,7 +807,7 @@
         <v>13305452</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
@@ -824,7 +824,7 @@
         <v>8948035</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -841,7 +841,7 @@
         <v>140931564</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -858,7 +858,7 @@
         <v>17896071</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -875,7 +875,7 @@
         <v>31318125</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -892,7 +892,7 @@
         <v>53688215</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -909,7 +909,7 @@
         <v>43365104</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -926,7 +926,7 @@
         <v>40213942</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -943,7 +943,7 @@
         <v>219201481</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -960,7 +960,7 @@
         <v>61220888</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
@@ -977,7 +977,7 @@
         <v>84680592</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -994,7 +994,7 @@
         <v>3625021</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>13464366</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>5390769</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>56510400</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>10</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>13</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>185663042</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>13</v>
       </c>
@@ -1113,7 +1113,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
@@ -1138,9 +1138,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFBA2FAA-95C5-423D-A8C0-3A912D67D407}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>12542</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>7598</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>14598</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1188,13 +1188,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5C2B8D5-A351-43B6-AB72-03AAE787B34B}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>37210000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>2610000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>35730000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>5706000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>5777000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1250,7 +1250,7 @@
         <v>3207000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>2595000</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>3123000</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>5222000</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>1900000</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>14250000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>

</xml_diff>